<commit_message>
Datos actualizados de costes de gráficas de 85 y 142 pág. Hoy me llegó la factura de Google Cloud y he ajustado el consumo de tokens de input/output para que cuadren con la factura recibida por Google Cloud, ya que mi benchmark calcula los tokens aproximados, ya que el sistema no los devuelve. Excel actualizado con los cálculos, para obtener el resultado exacto de la factura de Google Cloud.
</commit_message>
<xml_diff>
--- a/DataSet_142pag.xlsx
+++ b/DataSet_142pag.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Florian\Desktop\TFG_benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C49053-2C85-4529-93F0-898CA5162D62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005C7509-AD04-47A3-BAD3-D73451F666E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="2670" windowWidth="21600" windowHeight="11385" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RAG_Pinecone" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="189">
   <si>
     <t>ID</t>
   </si>
@@ -696,74 +696,175 @@
     <t>La respuesta generada es precisa y coincide con la respuesta real, indicando que el manual no contiene los códigos de color de pintura.</t>
   </si>
   <si>
-    <t>Tamaño del Documento</t>
-  </si>
-  <si>
-    <t>Tokens del PDF (Constante)</t>
-  </si>
-  <si>
-    <t>Input Tokens Reales (Fórmula en Excel)</t>
-  </si>
-  <si>
-    <t>10 Páginas</t>
-  </si>
-  <si>
-    <t>~4.700 tokens</t>
-  </si>
-  <si>
-    <t>4.700 + Input_Tokens_n8n</t>
-  </si>
-  <si>
-    <t>50 Páginas</t>
-  </si>
-  <si>
-    <t>~23.500 tokens</t>
-  </si>
-  <si>
-    <t>23.500 + Input_Tokens_n8n</t>
-  </si>
-  <si>
-    <t>100 Páginas</t>
-  </si>
-  <si>
-    <t>~47.000 tokens</t>
-  </si>
-  <si>
-    <t>47.000 + Input_Tokens_n8n</t>
-  </si>
-  <si>
-    <t>200 Páginas</t>
-  </si>
-  <si>
-    <t>~94.000 tokens</t>
-  </si>
-  <si>
-    <t>94.000 + Input_Tokens_n8n</t>
-  </si>
-  <si>
-    <t>300 Páginas</t>
-  </si>
-  <si>
-    <t>~141.000 tokens</t>
-  </si>
-  <si>
-    <t>(Ya tienes los datos reales del benchmark anterior)</t>
-  </si>
-  <si>
-    <t>&gt;aprox total</t>
-  </si>
-  <si>
     <t>27.176 tokens aprox tokens para PDF</t>
   </si>
   <si>
     <t>tienes menos texto este PDF</t>
+  </si>
+  <si>
+    <r>
+      <t>RAG Pinecone (Tarifa OpenAI):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">(40.386 / 1.000.000 * 0.417056) + (3.272 / 1.000.000 * 2.681684) = 0,0168 € + 0,0088 € = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0,0256 €</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>RAG Native (Tarifa Gemini Flash):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>(231.538 / 1.000.000 * 0.42) + (7.050 / 1.000.000 * 0.05) = 0,0972 € + 0,0003 € =</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve"> 0,0975 €</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Long Context (Tarifa Gemini Flash):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">(182.911 / 1.000.000 * 0.42) + (284 / 1.000.000 * 0.05) = 0,0768 € + 0,0001 € = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0,0769 €</t>
+    </r>
+  </si>
+  <si>
+    <t>Arquitectura</t>
+  </si>
+  <si>
+    <t>Coste Input (€)</t>
+  </si>
+  <si>
+    <t>Coste Output (€)</t>
+  </si>
+  <si>
+    <t>Coste Total (€)</t>
+  </si>
+  <si>
+    <t>RAG Pinecone</t>
+  </si>
+  <si>
+    <t>RAG Native</t>
+  </si>
+  <si>
+    <t>Long Context</t>
+  </si>
+  <si>
+    <t>&gt;coste total con 142 pag</t>
+  </si>
+  <si>
+    <t>coste factura= 0,27€ con 85pag + 0,20€ con 142 pag= 0,47€</t>
+  </si>
+  <si>
+    <r>
+      <t>Total Tokens Output</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(tokens ajustados para que cuadre con Factura de Google Cloud)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Total Tokens Input</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(tokens ajustados para que cuadre con Factura de Google Cloud)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -791,6 +892,55 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF0070C0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -800,7 +950,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -823,17 +973,58 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -989,6 +1180,153 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>77657</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>95328</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C004256F-608A-4F00-BAD3-287B5FBD37CB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="3905250"/>
+          <a:ext cx="10440857" cy="562053"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>77657</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>133428</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF119091-33A6-4554-9CF2-D44132C80CA7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4105275"/>
+          <a:ext cx="10440857" cy="562053"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2487482</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>104853</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C50AF9E-2B54-BAE2-36B3-88DDC43F2E2A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76200" y="5372100"/>
+          <a:ext cx="10440857" cy="562053"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1189,10 +1527,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N21"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:N23"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1236,7 +1574,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1280,7 +1618,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1324,7 +1662,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1368,7 +1706,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1412,7 +1750,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1456,7 +1794,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1500,7 +1838,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1544,7 +1882,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1588,7 +1926,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1632,7 +1970,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1676,7 +2014,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1720,7 +2058,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1764,7 +2102,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1808,7 +2146,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1852,7 +2190,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1896,7 +2234,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1940,7 +2278,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1984,7 +2322,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2028,7 +2366,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2072,7 +2410,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2116,17 +2454,28 @@
         <v>19</v>
       </c>
     </row>
+    <row r="23" spans="1:14">
+      <c r="H23">
+        <f>SUM(H2:H21)</f>
+        <v>40386</v>
+      </c>
+      <c r="I23">
+        <f>SUM(I2:I21)</f>
+        <v>3272</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N21"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:N24"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2170,7 +2519,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2214,7 +2563,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2258,7 +2607,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2302,7 +2651,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2346,7 +2695,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2390,7 +2739,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2434,7 +2783,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2478,7 +2827,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2522,7 +2871,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2566,7 +2915,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2610,7 +2959,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2654,7 +3003,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2698,7 +3047,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2742,7 +3091,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2786,7 +3135,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2830,7 +3179,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2874,7 +3223,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2918,7 +3267,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2962,7 +3311,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3006,7 +3355,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3050,30 +3399,48 @@
         <v>19</v>
       </c>
     </row>
+    <row r="24" spans="1:14">
+      <c r="H24">
+        <f>SUM(H2:H21)</f>
+        <v>540893</v>
+      </c>
+      <c r="I24">
+        <f>SUM(I2:I21)</f>
+        <v>54029</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N33"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:N35"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" customWidth="1"/>
+    <col min="3" max="3" width="45.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="31.85546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42.5703125" style="5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -3104,20 +3471,20 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="102">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="5" t="s">
         <v>134</v>
       </c>
       <c r="F2">
@@ -3148,20 +3515,20 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" ht="114.75">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="5" t="s">
         <v>136</v>
       </c>
       <c r="F3">
@@ -3192,20 +3559,20 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" ht="204">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="5" t="s">
         <v>138</v>
       </c>
       <c r="F4">
@@ -3236,20 +3603,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="153">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>24</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="5" t="s">
         <v>140</v>
       </c>
       <c r="F5">
@@ -3280,20 +3647,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="267.75">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>24</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="5" t="s">
         <v>142</v>
       </c>
       <c r="F6">
@@ -3324,20 +3691,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="216.75">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>24</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="5" t="s">
         <v>144</v>
       </c>
       <c r="F7">
@@ -3368,20 +3735,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="127.5">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>41</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>146</v>
       </c>
       <c r="F8">
@@ -3412,20 +3779,20 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="114.75">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>148</v>
       </c>
       <c r="F9">
@@ -3456,20 +3823,20 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" ht="102">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>41</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>149</v>
       </c>
       <c r="F10">
@@ -3500,20 +3867,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="127.5">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>151</v>
       </c>
       <c r="F11">
@@ -3544,20 +3911,20 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="204">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>58</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="5" t="s">
         <v>153</v>
       </c>
       <c r="F12">
@@ -3588,20 +3955,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ht="89.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>58</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="5" t="s">
         <v>155</v>
       </c>
       <c r="F13">
@@ -3632,20 +3999,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ht="127.5">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>58</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="5" t="s">
         <v>157</v>
       </c>
       <c r="F14">
@@ -3676,20 +4043,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ht="140.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="5" t="s">
         <v>159</v>
       </c>
       <c r="F15">
@@ -3720,20 +4087,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="51">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>75</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="5" t="s">
         <v>161</v>
       </c>
       <c r="F16">
@@ -3764,20 +4131,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" ht="153">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
         <v>75</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="5" t="s">
         <v>163</v>
       </c>
       <c r="F17">
@@ -3808,20 +4175,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" ht="89.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>75</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="5" t="s">
         <v>165</v>
       </c>
       <c r="F18">
@@ -3852,20 +4219,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" ht="204">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>75</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="5" t="s">
         <v>167</v>
       </c>
       <c r="F19">
@@ -3896,20 +4263,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" ht="409.5">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
         <v>92</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="5" t="s">
         <v>169</v>
       </c>
       <c r="F20">
@@ -3940,20 +4307,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" ht="255">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
         <v>92</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="5" t="s">
         <v>171</v>
       </c>
       <c r="F21">
@@ -3984,7 +4351,11 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14">
+      <c r="A24" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C24" s="6"/>
       <c r="H24">
         <f>SUM(H2:H21)</f>
         <v>7291</v>
@@ -3993,89 +4364,120 @@
         <f>SUM(I2:I21)</f>
         <v>2177</v>
       </c>
-      <c r="J24">
-        <f>H24+I24</f>
-        <v>9468</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="13.5" thickBot="1">
       <c r="I27" s="3" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B28" t="s">
         <v>173</v>
       </c>
-      <c r="C28" t="s">
+    </row>
+    <row r="28" spans="1:14" ht="51.75" thickBot="1">
+      <c r="A28" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="I28" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="D28" t="s">
-        <v>175</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B29" t="s">
-        <v>176</v>
-      </c>
-      <c r="C29" t="s">
-        <v>177</v>
-      </c>
-      <c r="D29" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B30" t="s">
-        <v>179</v>
-      </c>
-      <c r="C30" t="s">
-        <v>180</v>
-      </c>
-      <c r="D30" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B31" t="s">
+    </row>
+    <row r="29" spans="1:14" ht="26.25" thickBot="1">
+      <c r="A29" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="C31" t="s">
+      <c r="B29" s="8">
+        <v>40386</v>
+      </c>
+      <c r="C29" s="8">
+        <v>3272</v>
+      </c>
+      <c r="D29" s="9">
+        <v>1.6799999999999999E-2</v>
+      </c>
+      <c r="E29" s="9">
+        <v>8.8000000000000005E-3</v>
+      </c>
+      <c r="F29" s="10">
+        <v>2.5600000000000001E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="13.5" thickBot="1">
+      <c r="A30" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D31" t="s">
+      <c r="B30" s="8">
+        <v>231538</v>
+      </c>
+      <c r="C30" s="8">
+        <v>7050</v>
+      </c>
+      <c r="D30" s="9">
+        <v>9.7199999999999995E-2</v>
+      </c>
+      <c r="E30" s="9">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="F30" s="10">
+        <v>9.7500000000000003E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="26.25" thickBot="1">
+      <c r="A31" s="7" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B32" t="s">
+      <c r="B31" s="8">
+        <v>182911</v>
+      </c>
+      <c r="C31" s="11">
+        <v>284</v>
+      </c>
+      <c r="D31" s="9">
+        <v>7.6799999999999993E-2</v>
+      </c>
+      <c r="E31" s="9">
+        <v>1E-4</v>
+      </c>
+      <c r="F31" s="10">
+        <v>7.6899999999999996E-2</v>
+      </c>
+      <c r="H31" s="12">
+        <f>SUM(F29:F31)</f>
+        <v>0.2</v>
+      </c>
+      <c r="I31" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="C32" t="s">
+    </row>
+    <row r="35" spans="6:6">
+      <c r="F35" s="13" t="s">
         <v>186</v>
-      </c>
-      <c r="D32" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B33" t="s">
-        <v>188</v>
-      </c>
-      <c r="C33" t="s">
-        <v>189</v>
-      </c>
-      <c r="D33" t="s">
-        <v>190</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>